<commit_message>
Add new prototype of MemoryView + XRAM_View using VirtualScroller for pageless memory views
</commit_message>
<xml_diff>
--- a/fullständingt protokoll v3.06.xlsx
+++ b/fullständingt protokoll v3.06.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <fileVersion appName="Calc"/>
-  <workbookPr backupFile="false" showObjects="all" dateCompatibility="false"/>
+  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
     <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="4"/>
@@ -17,6 +17,7 @@
     <sheet name="övriga register" sheetId="7" state="visible" r:id="rId9"/>
     <sheet name="empty registers sheet" sheetId="8" state="visible" r:id="rId10"/>
     <sheet name="Sheet8" sheetId="9" state="visible" r:id="rId11"/>
+    <sheet name="sensor ADC lockup offsets" sheetId="10" state="visible" r:id="rId12"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
   <extLst>
@@ -28,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="525" uniqueCount="369">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="628" uniqueCount="450">
   <si>
     <t xml:space="preserve">alla requests är 9 bytes långa, börjar med 0x80 och slutar med EXOR CHECKSUM (som räknas ut endast av de 6 bytes payload)</t>
   </si>
@@ -57,7 +58,7 @@
     <t xml:space="preserve">respons</t>
   </si>
   <si>
-    <t xml:space="preserve">Intern ram adress</t>
+    <t xml:space="preserve">RAM adress</t>
   </si>
   <si>
     <t xml:space="preserve">cmd</t>
@@ -399,6 +400,18 @@
     <t xml:space="preserve">0x7ba1</t>
   </si>
   <si>
+    <t xml:space="preserve">read cmd 02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">write cmd 03</t>
+  </si>
+  <si>
+    <t xml:space="preserve">stored in flash</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Y</t>
+  </si>
+  <si>
     <t xml:space="preserve">Heat curve</t>
   </si>
   <si>
@@ -519,7 +532,7 @@
     <t xml:space="preserve">0x132E</t>
   </si>
   <si>
-    <t xml:space="preserve">Indoor temp setting </t>
+    <t xml:space="preserve">Indoor temp setting (GT5)</t>
   </si>
   <si>
     <t xml:space="preserve">0x0022</t>
@@ -540,6 +553,48 @@
     <t xml:space="preserve">GT3 Target value </t>
   </si>
   <si>
+    <t xml:space="preserve">0x003C</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0x1364</t>
+  </si>
+  <si>
+    <t xml:space="preserve">bestämmer vad extern styrning gör: 0(VP=on  EL=on  VV=on), 1(VP=off  EL=off  VV=off), 2(VP=on  EL=off  VV=off), 3(VP=on  EL=off  VV=on), 4(VP=on  EL=on  VV=off),</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0x003D</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0x1366</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Language setting</t>
+  </si>
+  <si>
+    <t xml:space="preserve">---</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0x003E</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0x1368</t>
+  </si>
+  <si>
+    <t xml:space="preserve">användas på meny typ 15 för visning av mystisk hårdkodad ’Adress’ sträng, troligtvis developer test, har ingen funktion</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0x41</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0x136E</t>
+  </si>
+  <si>
+    <t xml:space="preserve">16bit value ex. 3060 (dec)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Get/Set(temporary) firmware version</t>
+  </si>
+  <si>
     <t xml:space="preserve">0x0042</t>
   </si>
   <si>
@@ -567,6 +622,24 @@
     <t xml:space="preserve">Add heat activation time </t>
   </si>
   <si>
+    <t xml:space="preserve">0x65</t>
+  </si>
+  <si>
+    <t xml:space="preserve">calibration data??? </t>
+  </si>
+  <si>
+    <t xml:space="preserve">0x66</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0x67</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0x68</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0x69</t>
+  </si>
+  <si>
     <t xml:space="preserve">0x006B</t>
   </si>
   <si>
@@ -639,6 +712,12 @@
     <t xml:space="preserve">GT3 Off value </t>
   </si>
   <si>
+    <t xml:space="preserve">0x76</t>
+  </si>
+  <si>
+    <t xml:space="preserve">on/off state</t>
+  </si>
+  <si>
     <t xml:space="preserve">0x01FB</t>
   </si>
   <si>
@@ -663,7 +742,7 @@
     <t xml:space="preserve">0x16E8</t>
   </si>
   <si>
-    <t xml:space="preserve">Compresor </t>
+    <t xml:space="preserve">Compressor </t>
   </si>
   <si>
     <t xml:space="preserve">0x01FF</t>
@@ -720,6 +799,9 @@
     <t xml:space="preserve">Alarm </t>
   </si>
   <si>
+    <t xml:space="preserve">lockup index registry adress</t>
+  </si>
+  <si>
     <t xml:space="preserve">0x0209</t>
   </si>
   <si>
@@ -729,6 +811,9 @@
     <t xml:space="preserve">Radiator return [GT1] </t>
   </si>
   <si>
+    <t xml:space="preserve">1b64</t>
+  </si>
+  <si>
     <t xml:space="preserve">0x020A</t>
   </si>
   <si>
@@ -738,6 +823,9 @@
     <t xml:space="preserve">Outdoor [GT2] </t>
   </si>
   <si>
+    <t xml:space="preserve">1b66</t>
+  </si>
+  <si>
     <t xml:space="preserve">0x020B</t>
   </si>
   <si>
@@ -747,6 +835,9 @@
     <t xml:space="preserve">Hot water [GT3] </t>
   </si>
   <si>
+    <t xml:space="preserve">1b70</t>
+  </si>
+  <si>
     <t xml:space="preserve">0x020C</t>
   </si>
   <si>
@@ -756,6 +847,9 @@
     <t xml:space="preserve">Forward [GT4] </t>
   </si>
   <si>
+    <t xml:space="preserve">1b5e</t>
+  </si>
+  <si>
     <t xml:space="preserve">0x020D</t>
   </si>
   <si>
@@ -765,6 +859,9 @@
     <t xml:space="preserve">Room [GT5] </t>
   </si>
   <si>
+    <t xml:space="preserve">1b5c</t>
+  </si>
+  <si>
     <t xml:space="preserve">0x020E</t>
   </si>
   <si>
@@ -774,6 +871,9 @@
     <t xml:space="preserve">Compressor [GT6] </t>
   </si>
   <si>
+    <t xml:space="preserve">1b6e</t>
+  </si>
+  <si>
     <t xml:space="preserve">0x020F</t>
   </si>
   <si>
@@ -783,6 +883,9 @@
     <t xml:space="preserve">Heat fluid out [GT8] </t>
   </si>
   <si>
+    <t xml:space="preserve">1b6c</t>
+  </si>
+  <si>
     <t xml:space="preserve">0x0210</t>
   </si>
   <si>
@@ -792,6 +895,9 @@
     <t xml:space="preserve">Heat fluid in [GT9] </t>
   </si>
   <si>
+    <t xml:space="preserve">1bf3</t>
+  </si>
+  <si>
     <t xml:space="preserve">0x0211</t>
   </si>
   <si>
@@ -801,6 +907,9 @@
     <t xml:space="preserve">Cold fluid in [GT10] </t>
   </si>
   <si>
+    <t xml:space="preserve">1b6a</t>
+  </si>
+  <si>
     <t xml:space="preserve">0x0212</t>
   </si>
   <si>
@@ -810,6 +919,9 @@
     <t xml:space="preserve">Cold fluid out [GT11] </t>
   </si>
   <si>
+    <t xml:space="preserve">1b60</t>
+  </si>
+  <si>
     <t xml:space="preserve">0x0213</t>
   </si>
   <si>
@@ -817,6 +929,15 @@
   </si>
   <si>
     <t xml:space="preserve">External hot water [GT3x] </t>
+  </si>
+  <si>
+    <t xml:space="preserve">1b62</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Service Port Analog Input</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1b68</t>
   </si>
   <si>
     <t xml:space="preserve">Added heat timer in sec. </t>
@@ -925,6 +1046,9 @@
     <t xml:space="preserve">0x1EFC</t>
   </si>
   <si>
+    <t xml:space="preserve">ram adress =  0x0A6E</t>
+  </si>
+  <si>
     <t xml:space="preserve">Basindex 0x7bxx ersätt xx med koder nedan</t>
   </si>
   <si>
@@ -1099,15 +1223,12 @@
     <t xml:space="preserve">0x436</t>
   </si>
   <si>
+    <t xml:space="preserve">1b58</t>
+  </si>
+  <si>
     <t xml:space="preserve">0x3C</t>
   </si>
   <si>
-    <t xml:space="preserve">0x1364</t>
-  </si>
-  <si>
-    <t xml:space="preserve">bestämmer vad extern styrning gör: 0(VP=on  EL=on  VV=on), 1(VP=off  EL=off  VV=off), 2(VP=on  EL=off  VV=off), 3(VP=on  EL=off  VV=on), 4(VP=on  EL=on  VV=off),</t>
-  </si>
-  <si>
     <t xml:space="preserve">0x1FB</t>
   </si>
   <si>
@@ -1117,7 +1238,73 @@
     <t xml:space="preserve">0xA1C</t>
   </si>
   <si>
-    <t xml:space="preserve">value of register index @sysreg offset 0x446 (real adress 0x1b78)</t>
+    <t xml:space="preserve">0x</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0x7B5E</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0x9A8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RTC tid second</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0x7B5F</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0x9AA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RTC tid minute</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0x7B60</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0x9AC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RTC tid hour</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0x7B61</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0x9AE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RTC tid day</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0x7B62</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0x9B0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RTC tid month</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0x7B63</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0x9B2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RTC tid day of week</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0x7B64</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0x9B4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RtC tid year</t>
+  </si>
+  <si>
+    <t xml:space="preserve">value of register index @sysreg offset 0x447 (real adress 0x1b7A)</t>
   </si>
   <si>
     <t xml:space="preserve">RootScreen</t>
@@ -1132,10 +1319,67 @@
     <t xml:space="preserve">1F1C</t>
   </si>
   <si>
+    <t xml:space="preserve">1F3C</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1F5C</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1F5C(i ändra läge)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1F7C</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1F9C</t>
+  </si>
+  <si>
     <t xml:space="preserve">237C</t>
   </si>
   <si>
     <t xml:space="preserve">259C</t>
+  </si>
+  <si>
+    <t xml:space="preserve">26FC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">287C</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2CFC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2E9C</t>
+  </si>
+  <si>
+    <t xml:space="preserve">303C</t>
+  </si>
+  <si>
+    <t xml:space="preserve">333C</t>
+  </si>
+  <si>
+    <t xml:space="preserve">365C</t>
+  </si>
+  <si>
+    <t xml:space="preserve">36BC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">36FC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">371C</t>
+  </si>
+  <si>
+    <t xml:space="preserve">version</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0xF79C</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0xF7C6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0xF7E2</t>
   </si>
 </sst>
 </file>
@@ -1147,7 +1391,7 @@
     <numFmt numFmtId="165" formatCode="#,##0.00\ [$kr-41D];[RED]\-#,##0.00\ [$kr-41D]"/>
     <numFmt numFmtId="166" formatCode="@"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -1178,6 +1422,11 @@
       <sz val="10"/>
       <name val="Times New Roman"/>
       <family val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Courier New"/>
+      <family val="3"/>
     </font>
   </fonts>
   <fills count="3">
@@ -1229,7 +1478,7 @@
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="165" fontId="4" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="25">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1315,11 +1564,19 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -2481,6 +2738,60 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A3:B7"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="2" min="1" style="24" width="11.53"/>
+  </cols>
+  <sheetData>
+    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="24" t="s">
+        <v>446</v>
+      </c>
+      <c r="B3" s="24" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="24" t="n">
+        <v>3.021</v>
+      </c>
+      <c r="B5" s="24" t="s">
+        <v>447</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="24" t="n">
+        <v>3.06</v>
+      </c>
+      <c r="B6" s="24" t="s">
+        <v>448</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="24" t="n">
+        <v>3.12</v>
+      </c>
+      <c r="B7" s="24" t="s">
+        <v>449</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.025" bottom="1.025" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;A</oddHeader>
+    <oddFooter>&amp;CPage &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
@@ -2858,16 +3169,17 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H61"/>
+  <dimension ref="A1:I78"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.75" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="7" width="17.24"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="7" width="14.74"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="7" width="1.39"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="7" width="14.05"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="7" width="1.39"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="7" width="25.32"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="7" width="1.39"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="7" width="44.38"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="7" width="53.56"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2877,7 +3189,13 @@
       </c>
       <c r="B1" s="18"/>
       <c r="C1" s="17"/>
+      <c r="D1" s="7" t="s">
+        <v>123</v>
+      </c>
       <c r="E1" s="17"/>
+      <c r="F1" s="7" t="s">
+        <v>124</v>
+      </c>
       <c r="G1" s="17"/>
     </row>
     <row r="2" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2886,6 +3204,9 @@
       <c r="G2" s="17"/>
     </row>
     <row r="3" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="7" t="s">
+        <v>125</v>
+      </c>
       <c r="B3" s="7" t="s">
         <v>67</v>
       </c>
@@ -2903,7 +3224,7 @@
       </c>
     </row>
     <row r="4" customFormat="false" ht="7.45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="19"/>
+      <c r="A4" s="17"/>
       <c r="B4" s="14"/>
       <c r="C4" s="14"/>
       <c r="D4" s="14"/>
@@ -2913,6 +3234,9 @@
       <c r="H4" s="14"/>
     </row>
     <row r="5" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="7" t="s">
+        <v>126</v>
+      </c>
       <c r="B5" s="7" t="s">
         <v>24</v>
       </c>
@@ -2923,35 +3247,41 @@
       <c r="E5" s="14"/>
       <c r="G5" s="14"/>
       <c r="H5" s="7" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="7" t="s">
+        <v>126</v>
+      </c>
       <c r="B6" s="7" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="C6" s="14"/>
       <c r="D6" s="7" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="E6" s="14"/>
       <c r="G6" s="14"/>
       <c r="H6" s="7" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="7" t="s">
         <v>126</v>
       </c>
-    </row>
-    <row r="7" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="7" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="C7" s="14"/>
       <c r="D7" s="7" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="E7" s="14"/>
       <c r="G7" s="14"/>
       <c r="H7" s="7" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2965,12 +3295,12 @@
       </c>
       <c r="C9" s="14"/>
       <c r="D9" s="7" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="E9" s="14"/>
       <c r="G9" s="14"/>
       <c r="H9" s="7" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2979,54 +3309,54 @@
       </c>
       <c r="C10" s="14"/>
       <c r="D10" s="7" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="E10" s="14"/>
       <c r="G10" s="14"/>
       <c r="H10" s="20" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="7" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="C11" s="14"/>
       <c r="D11" s="7" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="E11" s="14"/>
       <c r="G11" s="14"/>
       <c r="H11" s="20" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="7" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="C12" s="14"/>
       <c r="D12" s="7" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="E12" s="14"/>
       <c r="G12" s="14"/>
       <c r="H12" s="20" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="7" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="C13" s="14"/>
       <c r="D13" s="7" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="E13" s="14"/>
       <c r="G13" s="14"/>
       <c r="H13" s="20" t="s">
-        <v>142</v>
+        <v>146</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3035,12 +3365,12 @@
       </c>
       <c r="C14" s="14"/>
       <c r="D14" s="7" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="E14" s="14"/>
       <c r="G14" s="14"/>
       <c r="H14" s="20" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3049,12 +3379,12 @@
       </c>
       <c r="C15" s="14"/>
       <c r="D15" s="7" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
       <c r="E15" s="14"/>
       <c r="G15" s="14"/>
       <c r="H15" s="20" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3063,96 +3393,96 @@
       </c>
       <c r="C16" s="14"/>
       <c r="D16" s="7" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="E16" s="14"/>
       <c r="G16" s="14"/>
       <c r="H16" s="20" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="7" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="C17" s="14"/>
       <c r="D17" s="7" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
       <c r="E17" s="14"/>
       <c r="G17" s="14"/>
       <c r="H17" s="20" t="s">
-        <v>151</v>
+        <v>155</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="7" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="C18" s="14"/>
       <c r="D18" s="7" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="E18" s="14"/>
       <c r="G18" s="14"/>
       <c r="H18" s="20" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="7" t="s">
-        <v>155</v>
+        <v>159</v>
       </c>
       <c r="C19" s="14"/>
       <c r="D19" s="7" t="s">
-        <v>156</v>
+        <v>160</v>
       </c>
       <c r="E19" s="14"/>
       <c r="G19" s="14"/>
       <c r="H19" s="20" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="7" t="s">
-        <v>158</v>
+        <v>162</v>
       </c>
       <c r="C20" s="14"/>
       <c r="D20" s="7" t="s">
-        <v>159</v>
+        <v>163</v>
       </c>
       <c r="E20" s="14"/>
       <c r="G20" s="14"/>
       <c r="H20" s="20" t="s">
-        <v>160</v>
+        <v>164</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="7" t="s">
-        <v>161</v>
+        <v>165</v>
       </c>
       <c r="C21" s="14"/>
       <c r="D21" s="7" t="s">
-        <v>162</v>
+        <v>166</v>
       </c>
       <c r="E21" s="14"/>
       <c r="G21" s="14"/>
       <c r="H21" s="20" t="s">
-        <v>163</v>
+        <v>167</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="7" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="C22" s="14"/>
       <c r="D22" s="7" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="E22" s="14"/>
       <c r="G22" s="14"/>
       <c r="H22" s="20" t="s">
-        <v>166</v>
+        <v>170</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3162,508 +3492,740 @@
     </row>
     <row r="24" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B24" s="7" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
       <c r="C24" s="14"/>
       <c r="D24" s="7" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
       <c r="E24" s="14"/>
       <c r="G24" s="14"/>
       <c r="H24" s="20" t="s">
-        <v>169</v>
+        <v>173</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B25" s="7" t="s">
-        <v>170</v>
-      </c>
       <c r="C25" s="14"/>
-      <c r="D25" s="7" t="s">
-        <v>171</v>
-      </c>
       <c r="E25" s="14"/>
       <c r="G25" s="14"/>
-      <c r="H25" s="20" t="s">
-        <v>172</v>
-      </c>
+      <c r="H25" s="20"/>
     </row>
     <row r="26" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B26" s="7" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="C26" s="14"/>
       <c r="D26" s="7" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="E26" s="14"/>
+      <c r="F26" s="7" t="s">
+        <v>113</v>
+      </c>
       <c r="G26" s="14"/>
-      <c r="H26" s="20" t="s">
-        <v>175</v>
+      <c r="H26" s="3" t="s">
+        <v>176</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B27" s="7" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="C27" s="14"/>
       <c r="D27" s="7" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="E27" s="14"/>
       <c r="G27" s="14"/>
       <c r="H27" s="20" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B28" s="7" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="C28" s="14"/>
-      <c r="D28" s="7" t="s">
-        <v>180</v>
-      </c>
       <c r="E28" s="14"/>
       <c r="G28" s="14"/>
-      <c r="H28" s="20" t="s">
+      <c r="H28" s="20"/>
+    </row>
+    <row r="29" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B29" s="7" t="s">
         <v>181</v>
-      </c>
-    </row>
-    <row r="29" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B29" s="7" t="s">
-        <v>182</v>
       </c>
       <c r="C29" s="14"/>
       <c r="D29" s="7" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="E29" s="14"/>
       <c r="G29" s="14"/>
       <c r="H29" s="20" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B30" s="7" t="s">
-        <v>185</v>
-      </c>
       <c r="C30" s="14"/>
-      <c r="D30" s="7" t="s">
-        <v>186</v>
-      </c>
       <c r="E30" s="14"/>
       <c r="G30" s="14"/>
-      <c r="H30" s="20" t="s">
-        <v>187</v>
-      </c>
+      <c r="H30" s="20"/>
     </row>
     <row r="31" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B31" s="7" t="s">
-        <v>188</v>
+        <v>184</v>
       </c>
       <c r="C31" s="14"/>
       <c r="D31" s="7" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="E31" s="14"/>
+      <c r="F31" s="7" t="s">
+        <v>186</v>
+      </c>
       <c r="G31" s="14"/>
       <c r="H31" s="20" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B32" s="7" t="s">
-        <v>191</v>
-      </c>
       <c r="C32" s="14"/>
-      <c r="D32" s="7" t="s">
-        <v>192</v>
-      </c>
       <c r="E32" s="14"/>
       <c r="G32" s="14"/>
-      <c r="H32" s="20" t="s">
-        <v>193</v>
-      </c>
+      <c r="H32" s="20"/>
     </row>
     <row r="33" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B33" s="7" t="s">
-        <v>194</v>
+        <v>188</v>
       </c>
       <c r="C33" s="14"/>
       <c r="D33" s="7" t="s">
-        <v>195</v>
+        <v>189</v>
       </c>
       <c r="E33" s="14"/>
       <c r="G33" s="14"/>
       <c r="H33" s="20" t="s">
-        <v>196</v>
+        <v>190</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B34" s="7" t="s">
-        <v>197</v>
+        <v>191</v>
       </c>
       <c r="C34" s="14"/>
       <c r="D34" s="7" t="s">
-        <v>198</v>
+        <v>192</v>
       </c>
       <c r="E34" s="14"/>
       <c r="G34" s="14"/>
       <c r="H34" s="20" t="s">
-        <v>199</v>
+        <v>193</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B35" s="7" t="s">
-        <v>200</v>
+        <v>194</v>
       </c>
       <c r="C35" s="14"/>
       <c r="D35" s="7" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
       <c r="E35" s="14"/>
       <c r="G35" s="14"/>
       <c r="H35" s="20" t="s">
-        <v>202</v>
+        <v>196</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C36" s="14"/>
       <c r="E36" s="14"/>
       <c r="G36" s="14"/>
+      <c r="H36" s="20"/>
     </row>
     <row r="37" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="7" t="s">
+        <v>126</v>
+      </c>
       <c r="B37" s="7" t="s">
-        <v>203</v>
+        <v>197</v>
       </c>
       <c r="C37" s="14"/>
-      <c r="D37" s="7" t="s">
-        <v>204</v>
-      </c>
       <c r="E37" s="14"/>
-      <c r="F37" s="7" t="s">
-        <v>92</v>
-      </c>
       <c r="G37" s="14"/>
-      <c r="H37" s="7" t="s">
-        <v>205</v>
+      <c r="H37" s="21" t="s">
+        <v>198</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="7" t="s">
+        <v>126</v>
+      </c>
+      <c r="B38" s="7" t="s">
+        <v>199</v>
+      </c>
       <c r="C38" s="14"/>
       <c r="E38" s="14"/>
       <c r="G38" s="14"/>
+      <c r="H38" s="21" t="s">
+        <v>198</v>
+      </c>
     </row>
     <row r="39" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="7" t="s">
+        <v>126</v>
+      </c>
       <c r="B39" s="7" t="s">
-        <v>206</v>
+        <v>200</v>
       </c>
       <c r="C39" s="14"/>
-      <c r="D39" s="7" t="s">
-        <v>207</v>
-      </c>
       <c r="E39" s="14"/>
-      <c r="F39" s="7" t="s">
-        <v>92</v>
-      </c>
       <c r="G39" s="14"/>
-      <c r="H39" s="20" t="s">
-        <v>208</v>
+      <c r="H39" s="21" t="s">
+        <v>198</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="7" t="s">
+        <v>126</v>
+      </c>
       <c r="B40" s="7" t="s">
-        <v>209</v>
+        <v>201</v>
       </c>
       <c r="C40" s="14"/>
-      <c r="D40" s="7" t="s">
-        <v>210</v>
-      </c>
       <c r="E40" s="14"/>
-      <c r="F40" s="7" t="s">
-        <v>92</v>
-      </c>
       <c r="G40" s="14"/>
-      <c r="H40" s="20" t="s">
-        <v>211</v>
+      <c r="H40" s="21" t="s">
+        <v>198</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="7" t="s">
+        <v>126</v>
+      </c>
       <c r="B41" s="7" t="s">
-        <v>212</v>
+        <v>202</v>
       </c>
       <c r="C41" s="14"/>
-      <c r="D41" s="7" t="s">
-        <v>213</v>
-      </c>
       <c r="E41" s="14"/>
-      <c r="F41" s="7" t="s">
-        <v>92</v>
-      </c>
       <c r="G41" s="14"/>
-      <c r="H41" s="20" t="s">
-        <v>214</v>
+      <c r="H41" s="21" t="s">
+        <v>198</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B42" s="7" t="s">
-        <v>215</v>
-      </c>
       <c r="C42" s="14"/>
-      <c r="D42" s="7" t="s">
-        <v>216</v>
-      </c>
       <c r="E42" s="14"/>
-      <c r="F42" s="7" t="s">
-        <v>92</v>
-      </c>
       <c r="G42" s="14"/>
-      <c r="H42" s="20" t="s">
-        <v>217</v>
-      </c>
+      <c r="H42" s="20"/>
     </row>
     <row r="43" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B43" s="7" t="s">
-        <v>218</v>
+        <v>203</v>
       </c>
       <c r="C43" s="14"/>
       <c r="D43" s="7" t="s">
-        <v>219</v>
+        <v>204</v>
       </c>
       <c r="E43" s="14"/>
-      <c r="F43" s="7" t="s">
-        <v>92</v>
-      </c>
       <c r="G43" s="14"/>
       <c r="H43" s="20" t="s">
-        <v>220</v>
+        <v>205</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B44" s="7" t="s">
-        <v>221</v>
+        <v>206</v>
       </c>
       <c r="C44" s="14"/>
       <c r="D44" s="7" t="s">
-        <v>222</v>
+        <v>207</v>
       </c>
       <c r="E44" s="14"/>
-      <c r="F44" s="7" t="s">
-        <v>92</v>
-      </c>
       <c r="G44" s="14"/>
-      <c r="H44" s="7" t="s">
-        <v>223</v>
+      <c r="H44" s="20" t="s">
+        <v>208</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B45" s="7" t="s">
-        <v>224</v>
+        <v>209</v>
       </c>
       <c r="C45" s="14"/>
       <c r="D45" s="7" t="s">
-        <v>225</v>
+        <v>210</v>
       </c>
       <c r="E45" s="14"/>
-      <c r="F45" s="7" t="s">
-        <v>92</v>
-      </c>
       <c r="G45" s="14"/>
-      <c r="H45" s="7" t="s">
-        <v>226</v>
+      <c r="H45" s="20" t="s">
+        <v>211</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B46" s="7" t="s">
-        <v>227</v>
+        <v>212</v>
       </c>
       <c r="C46" s="14"/>
       <c r="D46" s="7" t="s">
-        <v>228</v>
+        <v>213</v>
       </c>
       <c r="E46" s="14"/>
-      <c r="F46" s="7" t="s">
-        <v>92</v>
-      </c>
       <c r="G46" s="14"/>
-      <c r="H46" s="7" t="s">
-        <v>229</v>
+      <c r="H46" s="20" t="s">
+        <v>214</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B47" s="7" t="s">
+        <v>215</v>
+      </c>
       <c r="C47" s="14"/>
+      <c r="D47" s="7" t="s">
+        <v>216</v>
+      </c>
       <c r="E47" s="14"/>
       <c r="G47" s="14"/>
+      <c r="H47" s="20" t="s">
+        <v>217</v>
+      </c>
     </row>
     <row r="48" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B48" s="7" t="s">
-        <v>230</v>
+        <v>218</v>
       </c>
       <c r="C48" s="14"/>
       <c r="D48" s="7" t="s">
-        <v>231</v>
+        <v>219</v>
       </c>
       <c r="E48" s="14"/>
       <c r="G48" s="14"/>
       <c r="H48" s="20" t="s">
-        <v>232</v>
+        <v>220</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B49" s="7" t="s">
-        <v>233</v>
+        <v>221</v>
       </c>
       <c r="C49" s="14"/>
       <c r="D49" s="7" t="s">
-        <v>234</v>
+        <v>222</v>
       </c>
       <c r="E49" s="14"/>
       <c r="G49" s="14"/>
       <c r="H49" s="20" t="s">
-        <v>235</v>
+        <v>223</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B50" s="7" t="s">
-        <v>236</v>
+        <v>224</v>
       </c>
       <c r="C50" s="14"/>
       <c r="D50" s="7" t="s">
-        <v>237</v>
+        <v>225</v>
       </c>
       <c r="E50" s="14"/>
       <c r="G50" s="14"/>
       <c r="H50" s="20" t="s">
-        <v>238</v>
+        <v>226</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B51" s="7" t="s">
-        <v>239</v>
-      </c>
       <c r="C51" s="14"/>
-      <c r="D51" s="7" t="s">
-        <v>240</v>
-      </c>
       <c r="E51" s="14"/>
       <c r="G51" s="14"/>
-      <c r="H51" s="20" t="s">
-        <v>241</v>
-      </c>
     </row>
     <row r="52" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A52" s="7" t="s">
+        <v>126</v>
+      </c>
       <c r="B52" s="7" t="s">
-        <v>242</v>
+        <v>227</v>
       </c>
       <c r="C52" s="14"/>
-      <c r="D52" s="7" t="s">
-        <v>243</v>
-      </c>
       <c r="E52" s="14"/>
       <c r="G52" s="14"/>
-      <c r="H52" s="20" t="s">
-        <v>244</v>
+      <c r="H52" s="7" t="s">
+        <v>228</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B53" s="7" t="s">
-        <v>245</v>
-      </c>
       <c r="C53" s="14"/>
-      <c r="D53" s="7" t="s">
-        <v>246</v>
-      </c>
       <c r="E53" s="14"/>
       <c r="G53" s="14"/>
-      <c r="H53" s="20" t="s">
-        <v>247</v>
-      </c>
     </row>
     <row r="54" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B54" s="7" t="s">
-        <v>248</v>
+        <v>229</v>
       </c>
       <c r="C54" s="14"/>
       <c r="D54" s="7" t="s">
-        <v>249</v>
+        <v>230</v>
       </c>
       <c r="E54" s="14"/>
+      <c r="F54" s="7" t="s">
+        <v>92</v>
+      </c>
       <c r="G54" s="14"/>
-      <c r="H54" s="20" t="s">
-        <v>250</v>
+      <c r="H54" s="7" t="s">
+        <v>231</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B55" s="7" t="s">
-        <v>251</v>
-      </c>
       <c r="C55" s="14"/>
-      <c r="D55" s="7" t="s">
-        <v>252</v>
-      </c>
       <c r="E55" s="14"/>
       <c r="G55" s="14"/>
-      <c r="H55" s="20" t="s">
-        <v>253</v>
-      </c>
     </row>
     <row r="56" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B56" s="7" t="s">
-        <v>254</v>
+        <v>232</v>
       </c>
       <c r="C56" s="14"/>
       <c r="D56" s="7" t="s">
-        <v>255</v>
+        <v>233</v>
       </c>
       <c r="E56" s="14"/>
+      <c r="F56" s="7" t="s">
+        <v>92</v>
+      </c>
       <c r="G56" s="14"/>
       <c r="H56" s="20" t="s">
-        <v>256</v>
+        <v>234</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B57" s="7" t="s">
-        <v>257</v>
+        <v>235</v>
       </c>
       <c r="C57" s="14"/>
       <c r="D57" s="7" t="s">
-        <v>258</v>
+        <v>236</v>
       </c>
       <c r="E57" s="14"/>
+      <c r="F57" s="7" t="s">
+        <v>92</v>
+      </c>
       <c r="G57" s="14"/>
       <c r="H57" s="20" t="s">
-        <v>259</v>
+        <v>237</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B58" s="7" t="s">
-        <v>260</v>
+        <v>238</v>
       </c>
       <c r="C58" s="14"/>
       <c r="D58" s="7" t="s">
-        <v>261</v>
+        <v>239</v>
       </c>
       <c r="E58" s="14"/>
+      <c r="F58" s="7" t="s">
+        <v>92</v>
+      </c>
       <c r="G58" s="14"/>
       <c r="H58" s="20" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="59" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B59" s="7" t="s">
+        <v>241</v>
+      </c>
+      <c r="C59" s="14"/>
+      <c r="D59" s="7" t="s">
+        <v>242</v>
+      </c>
+      <c r="E59" s="14"/>
+      <c r="F59" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="G59" s="14"/>
+      <c r="H59" s="20" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="60" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B60" s="7" t="s">
+        <v>244</v>
+      </c>
+      <c r="C60" s="14"/>
+      <c r="D60" s="7" t="s">
+        <v>245</v>
+      </c>
+      <c r="E60" s="14"/>
+      <c r="F60" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="G60" s="14"/>
+      <c r="H60" s="20" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="61" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B61" s="7" t="s">
+        <v>247</v>
+      </c>
+      <c r="C61" s="14"/>
+      <c r="D61" s="7" t="s">
+        <v>248</v>
+      </c>
+      <c r="E61" s="14"/>
+      <c r="F61" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="G61" s="14"/>
+      <c r="H61" s="7" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="62" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B62" s="7" t="s">
+        <v>250</v>
+      </c>
+      <c r="C62" s="14"/>
+      <c r="D62" s="7" t="s">
+        <v>251</v>
+      </c>
+      <c r="E62" s="14"/>
+      <c r="F62" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="G62" s="14"/>
+      <c r="H62" s="7" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="63" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B63" s="7" t="s">
+        <v>253</v>
+      </c>
+      <c r="C63" s="14"/>
+      <c r="D63" s="7" t="s">
+        <v>254</v>
+      </c>
+      <c r="E63" s="14"/>
+      <c r="F63" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="G63" s="14"/>
+      <c r="H63" s="7" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="64" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C64" s="14"/>
+      <c r="E64" s="14"/>
+      <c r="G64" s="14"/>
+      <c r="I64" s="0" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="65" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B65" s="7" t="s">
+        <v>257</v>
+      </c>
+      <c r="C65" s="14"/>
+      <c r="D65" s="7" t="s">
+        <v>258</v>
+      </c>
+      <c r="E65" s="14"/>
+      <c r="G65" s="14"/>
+      <c r="H65" s="20" t="s">
+        <v>259</v>
+      </c>
+      <c r="I65" s="0" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="66" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B66" s="7" t="s">
+        <v>261</v>
+      </c>
+      <c r="C66" s="14"/>
+      <c r="D66" s="7" t="s">
         <v>262</v>
       </c>
-    </row>
-    <row r="59" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C59" s="14"/>
-      <c r="E59" s="14"/>
-      <c r="G59" s="14"/>
-    </row>
-    <row r="60" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C60" s="14"/>
-      <c r="E60" s="14"/>
-      <c r="G60" s="14"/>
-    </row>
-    <row r="61" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C61" s="14"/>
-      <c r="E61" s="14"/>
-      <c r="G61" s="14"/>
+      <c r="E66" s="14"/>
+      <c r="G66" s="14"/>
+      <c r="H66" s="20" t="s">
+        <v>263</v>
+      </c>
+      <c r="I66" s="0" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="67" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B67" s="7" t="s">
+        <v>265</v>
+      </c>
+      <c r="C67" s="14"/>
+      <c r="D67" s="7" t="s">
+        <v>266</v>
+      </c>
+      <c r="E67" s="14"/>
+      <c r="G67" s="14"/>
+      <c r="H67" s="20" t="s">
+        <v>267</v>
+      </c>
+      <c r="I67" s="0" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="68" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B68" s="7" t="s">
+        <v>269</v>
+      </c>
+      <c r="C68" s="14"/>
+      <c r="D68" s="7" t="s">
+        <v>270</v>
+      </c>
+      <c r="E68" s="14"/>
+      <c r="G68" s="14"/>
+      <c r="H68" s="20" t="s">
+        <v>271</v>
+      </c>
+      <c r="I68" s="0" t="s">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="69" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B69" s="7" t="s">
+        <v>273</v>
+      </c>
+      <c r="C69" s="14"/>
+      <c r="D69" s="7" t="s">
+        <v>274</v>
+      </c>
+      <c r="E69" s="14"/>
+      <c r="G69" s="14"/>
+      <c r="H69" s="20" t="s">
+        <v>275</v>
+      </c>
+      <c r="I69" s="0" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="70" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B70" s="7" t="s">
+        <v>277</v>
+      </c>
+      <c r="C70" s="14"/>
+      <c r="D70" s="7" t="s">
+        <v>278</v>
+      </c>
+      <c r="E70" s="14"/>
+      <c r="G70" s="14"/>
+      <c r="H70" s="20" t="s">
+        <v>279</v>
+      </c>
+      <c r="I70" s="0" t="s">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="71" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B71" s="7" t="s">
+        <v>281</v>
+      </c>
+      <c r="C71" s="14"/>
+      <c r="D71" s="7" t="s">
+        <v>282</v>
+      </c>
+      <c r="E71" s="14"/>
+      <c r="G71" s="14"/>
+      <c r="H71" s="20" t="s">
+        <v>283</v>
+      </c>
+      <c r="I71" s="0" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="72" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B72" s="7" t="s">
+        <v>285</v>
+      </c>
+      <c r="C72" s="14"/>
+      <c r="D72" s="7" t="s">
+        <v>286</v>
+      </c>
+      <c r="E72" s="14"/>
+      <c r="G72" s="14"/>
+      <c r="H72" s="20" t="s">
+        <v>287</v>
+      </c>
+      <c r="I72" s="0" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="73" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B73" s="7" t="s">
+        <v>289</v>
+      </c>
+      <c r="C73" s="14"/>
+      <c r="D73" s="7" t="s">
+        <v>290</v>
+      </c>
+      <c r="E73" s="14"/>
+      <c r="G73" s="14"/>
+      <c r="H73" s="20" t="s">
+        <v>291</v>
+      </c>
+      <c r="I73" s="0" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="74" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B74" s="7" t="s">
+        <v>293</v>
+      </c>
+      <c r="C74" s="14"/>
+      <c r="D74" s="7" t="s">
+        <v>294</v>
+      </c>
+      <c r="E74" s="14"/>
+      <c r="G74" s="14"/>
+      <c r="H74" s="20" t="s">
+        <v>295</v>
+      </c>
+      <c r="I74" s="0" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="75" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B75" s="7" t="s">
+        <v>297</v>
+      </c>
+      <c r="C75" s="14"/>
+      <c r="D75" s="7" t="s">
+        <v>298</v>
+      </c>
+      <c r="E75" s="14"/>
+      <c r="G75" s="14"/>
+      <c r="H75" s="20" t="s">
+        <v>299</v>
+      </c>
+      <c r="I75" s="0" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="76" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C76" s="14"/>
+      <c r="E76" s="14"/>
+      <c r="G76" s="14"/>
+    </row>
+    <row r="77" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C77" s="14"/>
+      <c r="E77" s="14"/>
+      <c r="G77" s="14"/>
+      <c r="H77" s="7" t="s">
+        <v>301</v>
+      </c>
+      <c r="I77" s="0" t="s">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="78" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C78" s="14"/>
+      <c r="E78" s="14"/>
+      <c r="G78" s="14"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -3749,23 +4311,23 @@
       <c r="E5" s="14"/>
       <c r="F5" s="0"/>
       <c r="G5" s="14"/>
-      <c r="H5" s="21" t="s">
-        <v>263</v>
+      <c r="H5" s="22" t="s">
+        <v>303</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="7" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="C6" s="14"/>
       <c r="D6" s="7" t="s">
-        <v>264</v>
+        <v>304</v>
       </c>
       <c r="E6" s="14"/>
       <c r="F6" s="0"/>
       <c r="G6" s="14"/>
-      <c r="H6" s="21" t="s">
-        <v>265</v>
+      <c r="H6" s="22" t="s">
+        <v>305</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3777,7 +4339,7 @@
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="7" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="C8" s="14"/>
       <c r="D8" s="7" t="s">
@@ -3786,8 +4348,8 @@
       <c r="E8" s="14"/>
       <c r="F8" s="0"/>
       <c r="G8" s="14"/>
-      <c r="H8" s="22" t="s">
-        <v>266</v>
+      <c r="H8" s="23" t="s">
+        <v>306</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3799,17 +4361,17 @@
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="7" t="s">
-        <v>267</v>
+        <v>307</v>
       </c>
       <c r="C10" s="14"/>
       <c r="D10" s="7" t="s">
-        <v>268</v>
+        <v>308</v>
       </c>
       <c r="E10" s="14"/>
       <c r="F10" s="0"/>
       <c r="G10" s="14"/>
       <c r="H10" s="7" t="s">
-        <v>269</v>
+        <v>309</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3821,62 +4383,62 @@
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="7" t="s">
-        <v>270</v>
+        <v>310</v>
       </c>
       <c r="C12" s="14"/>
       <c r="D12" s="7" t="s">
-        <v>271</v>
+        <v>311</v>
       </c>
       <c r="E12" s="14"/>
       <c r="F12" s="0"/>
       <c r="G12" s="14"/>
-      <c r="H12" s="22" t="s">
-        <v>272</v>
+      <c r="H12" s="23" t="s">
+        <v>312</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="7" t="s">
-        <v>273</v>
+        <v>313</v>
       </c>
       <c r="C13" s="14"/>
       <c r="D13" s="7" t="s">
-        <v>274</v>
+        <v>314</v>
       </c>
       <c r="E13" s="14"/>
       <c r="F13" s="0"/>
       <c r="G13" s="14"/>
-      <c r="H13" s="22" t="s">
-        <v>275</v>
+      <c r="H13" s="23" t="s">
+        <v>315</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="7" t="s">
-        <v>276</v>
+        <v>316</v>
       </c>
       <c r="C14" s="14"/>
       <c r="D14" s="7" t="s">
-        <v>277</v>
+        <v>317</v>
       </c>
       <c r="E14" s="14"/>
       <c r="F14" s="0"/>
       <c r="G14" s="14"/>
-      <c r="H14" s="22" t="s">
-        <v>278</v>
+      <c r="H14" s="23" t="s">
+        <v>318</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="7" t="s">
-        <v>279</v>
+        <v>319</v>
       </c>
       <c r="C15" s="14"/>
       <c r="D15" s="7" t="s">
-        <v>280</v>
+        <v>320</v>
       </c>
       <c r="E15" s="14"/>
       <c r="F15" s="0"/>
       <c r="G15" s="14"/>
-      <c r="H15" s="22" t="s">
-        <v>281</v>
+      <c r="H15" s="23" t="s">
+        <v>321</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3975,10 +4537,10 @@
       </c>
       <c r="I3" s="16"/>
       <c r="J3" s="7" t="s">
-        <v>282</v>
+        <v>322</v>
       </c>
       <c r="K3" s="7" t="s">
-        <v>283</v>
+        <v>323</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="7.45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4002,11 +4564,11 @@
     </row>
     <row r="6" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="7" t="s">
-        <v>284</v>
+        <v>324</v>
       </c>
       <c r="C6" s="14"/>
       <c r="D6" s="7" t="s">
-        <v>285</v>
+        <v>325</v>
       </c>
       <c r="E6" s="14"/>
       <c r="F6" s="7" t="s">
@@ -4014,14 +4576,14 @@
       </c>
       <c r="G6" s="14"/>
       <c r="H6" s="3" t="s">
-        <v>286</v>
+        <v>326</v>
       </c>
       <c r="I6" s="16"/>
       <c r="J6" s="7" t="s">
-        <v>287</v>
+        <v>327</v>
       </c>
       <c r="K6" s="7" t="s">
-        <v>288</v>
+        <v>328</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4032,23 +4594,23 @@
     </row>
     <row r="8" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="17" t="s">
-        <v>289</v>
+        <v>329</v>
       </c>
       <c r="C8" s="14"/>
       <c r="D8" s="17" t="s">
-        <v>271</v>
+        <v>311</v>
       </c>
       <c r="E8" s="14"/>
       <c r="F8" s="17" t="s">
-        <v>290</v>
+        <v>330</v>
       </c>
       <c r="G8" s="14"/>
       <c r="H8" s="15" t="s">
-        <v>291</v>
+        <v>331</v>
       </c>
       <c r="I8" s="16"/>
       <c r="J8" s="7" t="s">
-        <v>292</v>
+        <v>332</v>
       </c>
       <c r="K8" s="7" t="s">
         <v>25</v>
@@ -4056,23 +4618,23 @@
     </row>
     <row r="9" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="7" t="s">
-        <v>293</v>
+        <v>333</v>
       </c>
       <c r="C9" s="14"/>
       <c r="D9" s="7" t="s">
-        <v>294</v>
+        <v>334</v>
       </c>
       <c r="E9" s="14"/>
       <c r="F9" s="7" t="s">
-        <v>295</v>
+        <v>335</v>
       </c>
       <c r="G9" s="14"/>
       <c r="H9" s="3" t="s">
-        <v>296</v>
+        <v>336</v>
       </c>
       <c r="I9" s="16"/>
       <c r="J9" s="7" t="s">
-        <v>297</v>
+        <v>337</v>
       </c>
       <c r="K9" s="7" t="s">
         <v>25</v>
@@ -4173,7 +4735,9 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="7" width="25.32"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="7" width="1.39"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="3" width="44.38"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="29" min="9" style="0" width="3.58"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="9" style="0" width="3.58"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="0" width="3.75"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="29" min="18" style="0" width="3.58"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4185,6 +4749,9 @@
       <c r="C1" s="17"/>
       <c r="E1" s="17"/>
       <c r="G1" s="17"/>
+      <c r="H1" s="3" t="s">
+        <v>338</v>
+      </c>
       <c r="I1" s="5" t="s">
         <v>70</v>
       </c>
@@ -4202,7 +4769,7 @@
       <c r="E2" s="17"/>
       <c r="G2" s="17"/>
       <c r="I2" s="5" t="s">
-        <v>298</v>
+        <v>339</v>
       </c>
       <c r="J2" s="5"/>
       <c r="K2" s="5"/>
@@ -4331,220 +4898,220 @@
       </c>
       <c r="E5" s="14"/>
       <c r="F5" s="7" t="s">
-        <v>299</v>
+        <v>340</v>
       </c>
       <c r="G5" s="14"/>
       <c r="H5" s="3" t="s">
-        <v>300</v>
+        <v>341</v>
       </c>
       <c r="I5" s="7"/>
       <c r="J5" s="7" t="s">
-        <v>301</v>
+        <v>342</v>
       </c>
       <c r="K5" s="7"/>
       <c r="L5" s="7" t="s">
-        <v>302</v>
+        <v>343</v>
       </c>
       <c r="M5" s="7"/>
       <c r="N5" s="7" t="s">
-        <v>303</v>
+        <v>344</v>
       </c>
       <c r="O5" s="7"/>
       <c r="P5" s="7" t="s">
-        <v>304</v>
+        <v>345</v>
       </c>
       <c r="Q5" s="7"/>
       <c r="R5" s="7" t="s">
-        <v>305</v>
+        <v>346</v>
       </c>
       <c r="S5" s="7"/>
       <c r="T5" s="7" t="s">
-        <v>306</v>
+        <v>347</v>
       </c>
       <c r="U5" s="7"/>
       <c r="V5" s="7" t="s">
-        <v>307</v>
+        <v>348</v>
       </c>
       <c r="W5" s="7"/>
       <c r="X5" s="7" t="s">
-        <v>308</v>
+        <v>349</v>
       </c>
       <c r="Y5" s="7"/>
       <c r="Z5" s="7" t="s">
-        <v>309</v>
+        <v>350</v>
       </c>
       <c r="AA5" s="7"/>
       <c r="AB5" s="7" t="s">
-        <v>310</v>
+        <v>351</v>
       </c>
       <c r="AC5" s="7"/>
     </row>
     <row r="6" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="7" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="C6" s="14"/>
       <c r="D6" s="7" t="s">
-        <v>311</v>
+        <v>352</v>
       </c>
       <c r="E6" s="14"/>
       <c r="F6" s="7" t="s">
-        <v>299</v>
+        <v>340</v>
       </c>
       <c r="G6" s="14"/>
       <c r="H6" s="3" t="s">
-        <v>312</v>
+        <v>353</v>
       </c>
       <c r="I6" s="7" t="s">
-        <v>313</v>
+        <v>354</v>
       </c>
       <c r="J6" s="7"/>
       <c r="K6" s="7" t="s">
-        <v>314</v>
+        <v>355</v>
       </c>
       <c r="L6" s="7"/>
       <c r="M6" s="7" t="s">
-        <v>315</v>
+        <v>356</v>
       </c>
       <c r="N6" s="7"/>
       <c r="O6" s="7" t="s">
-        <v>316</v>
+        <v>357</v>
       </c>
       <c r="P6" s="7"/>
       <c r="Q6" s="7" t="s">
-        <v>317</v>
+        <v>358</v>
       </c>
       <c r="R6" s="7"/>
       <c r="S6" s="7" t="s">
-        <v>318</v>
+        <v>359</v>
       </c>
       <c r="T6" s="7"/>
       <c r="U6" s="7" t="s">
-        <v>319</v>
+        <v>360</v>
       </c>
       <c r="V6" s="7"/>
       <c r="W6" s="7" t="s">
-        <v>320</v>
+        <v>361</v>
       </c>
       <c r="X6" s="7"/>
       <c r="Y6" s="7" t="s">
-        <v>321</v>
+        <v>362</v>
       </c>
       <c r="Z6" s="7"/>
       <c r="AA6" s="7" t="s">
-        <v>322</v>
+        <v>363</v>
       </c>
       <c r="AB6" s="7"/>
       <c r="AC6" s="7" t="s">
-        <v>323</v>
+        <v>364</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="7" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="C7" s="14"/>
       <c r="D7" s="7" t="s">
-        <v>324</v>
+        <v>365</v>
       </c>
       <c r="E7" s="14"/>
       <c r="F7" s="7" t="s">
-        <v>299</v>
+        <v>340</v>
       </c>
       <c r="G7" s="14"/>
       <c r="H7" s="3" t="s">
-        <v>325</v>
+        <v>366</v>
       </c>
       <c r="I7" s="7"/>
       <c r="J7" s="7" t="s">
-        <v>326</v>
+        <v>367</v>
       </c>
       <c r="K7" s="7"/>
       <c r="L7" s="7" t="s">
-        <v>327</v>
+        <v>368</v>
       </c>
       <c r="M7" s="7"/>
       <c r="N7" s="7" t="s">
-        <v>328</v>
+        <v>369</v>
       </c>
       <c r="O7" s="7"/>
       <c r="P7" s="7" t="s">
-        <v>329</v>
+        <v>370</v>
       </c>
       <c r="Q7" s="7"/>
       <c r="R7" s="7" t="s">
-        <v>330</v>
+        <v>371</v>
       </c>
       <c r="S7" s="7"/>
       <c r="T7" s="7" t="s">
-        <v>331</v>
+        <v>372</v>
       </c>
       <c r="U7" s="7"/>
       <c r="V7" s="7" t="s">
-        <v>332</v>
+        <v>373</v>
       </c>
       <c r="W7" s="7"/>
       <c r="X7" s="7" t="s">
-        <v>333</v>
+        <v>374</v>
       </c>
       <c r="Y7" s="7"/>
       <c r="Z7" s="7" t="s">
-        <v>334</v>
+        <v>375</v>
       </c>
       <c r="AA7" s="7"/>
       <c r="AB7" s="7" t="s">
-        <v>335</v>
+        <v>376</v>
       </c>
       <c r="AC7" s="7"/>
     </row>
     <row r="8" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="7" t="s">
-        <v>336</v>
+        <v>377</v>
       </c>
       <c r="C8" s="14"/>
       <c r="D8" s="7" t="s">
-        <v>337</v>
+        <v>378</v>
       </c>
       <c r="E8" s="14"/>
       <c r="F8" s="7" t="s">
-        <v>299</v>
+        <v>340</v>
       </c>
       <c r="G8" s="14"/>
       <c r="H8" s="3" t="s">
-        <v>338</v>
+        <v>379</v>
       </c>
       <c r="I8" s="0" t="s">
-        <v>339</v>
+        <v>380</v>
       </c>
       <c r="K8" s="0" t="s">
-        <v>340</v>
+        <v>381</v>
       </c>
       <c r="M8" s="0" t="s">
-        <v>341</v>
+        <v>382</v>
       </c>
       <c r="O8" s="0" t="s">
-        <v>342</v>
+        <v>383</v>
       </c>
       <c r="Q8" s="0" t="s">
-        <v>343</v>
+        <v>384</v>
       </c>
       <c r="S8" s="0" t="s">
-        <v>344</v>
+        <v>385</v>
       </c>
       <c r="U8" s="0" t="s">
-        <v>345</v>
+        <v>386</v>
       </c>
       <c r="W8" s="0" t="s">
-        <v>346</v>
+        <v>387</v>
       </c>
       <c r="Y8" s="0" t="s">
-        <v>347</v>
+        <v>388</v>
       </c>
       <c r="AA8" s="0" t="s">
-        <v>348</v>
+        <v>389</v>
       </c>
       <c r="AC8" s="0" t="s">
-        <v>349</v>
+        <v>390</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4691,7 +5258,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:K22"/>
+  <dimension ref="A1:K26"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.75" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="7" width="14.74"/>
@@ -4737,10 +5304,10 @@
         <v>6</v>
       </c>
       <c r="J3" s="7" t="s">
-        <v>282</v>
+        <v>322</v>
       </c>
       <c r="K3" s="7" t="s">
-        <v>283</v>
+        <v>323</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="7.45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4759,23 +5326,23 @@
     <row r="5" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="19"/>
       <c r="B5" s="17" t="s">
-        <v>350</v>
+        <v>391</v>
       </c>
       <c r="C5" s="14"/>
       <c r="D5" s="17" t="s">
-        <v>271</v>
+        <v>311</v>
       </c>
       <c r="E5" s="14"/>
       <c r="F5" s="17" t="s">
-        <v>290</v>
+        <v>330</v>
       </c>
       <c r="G5" s="14"/>
       <c r="H5" s="15" t="s">
-        <v>291</v>
+        <v>331</v>
       </c>
       <c r="I5" s="15"/>
       <c r="J5" s="7" t="s">
-        <v>292</v>
+        <v>332</v>
       </c>
       <c r="K5" s="7" t="s">
         <v>25</v>
@@ -4783,22 +5350,22 @@
     </row>
     <row r="6" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="7" t="s">
-        <v>351</v>
+        <v>392</v>
       </c>
       <c r="C6" s="14"/>
       <c r="D6" s="7" t="s">
-        <v>294</v>
+        <v>334</v>
       </c>
       <c r="E6" s="14"/>
       <c r="F6" s="7" t="s">
-        <v>295</v>
+        <v>335</v>
       </c>
       <c r="G6" s="14"/>
       <c r="H6" s="3" t="s">
-        <v>296</v>
+        <v>336</v>
       </c>
       <c r="J6" s="7" t="s">
-        <v>297</v>
+        <v>337</v>
       </c>
       <c r="K6" s="7" t="s">
         <v>25</v>
@@ -4811,11 +5378,11 @@
     </row>
     <row r="8" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="7" t="s">
-        <v>352</v>
+        <v>393</v>
       </c>
       <c r="C8" s="14"/>
       <c r="D8" s="7" t="s">
-        <v>274</v>
+        <v>314</v>
       </c>
       <c r="E8" s="14"/>
       <c r="F8" s="7" t="s">
@@ -4823,12 +5390,12 @@
       </c>
       <c r="G8" s="14"/>
       <c r="H8" s="3" t="s">
-        <v>353</v>
+        <v>394</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="7" t="s">
-        <v>354</v>
+        <v>395</v>
       </c>
       <c r="C9" s="14"/>
       <c r="D9" s="7" t="s">
@@ -4845,11 +5412,11 @@
     </row>
     <row r="10" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="7" t="s">
-        <v>355</v>
+        <v>396</v>
       </c>
       <c r="C10" s="14"/>
       <c r="D10" s="7" t="s">
-        <v>285</v>
+        <v>397</v>
       </c>
       <c r="E10" s="14"/>
       <c r="F10" s="7" t="s">
@@ -4857,13 +5424,13 @@
       </c>
       <c r="G10" s="14"/>
       <c r="H10" s="3" t="s">
-        <v>286</v>
+        <v>326</v>
       </c>
       <c r="J10" s="7" t="s">
-        <v>287</v>
+        <v>327</v>
       </c>
       <c r="K10" s="7" t="s">
-        <v>288</v>
+        <v>328</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4878,11 +5445,11 @@
     </row>
     <row r="13" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="7" t="s">
-        <v>356</v>
+        <v>398</v>
       </c>
       <c r="C13" s="14"/>
       <c r="D13" s="7" t="s">
-        <v>357</v>
+        <v>175</v>
       </c>
       <c r="E13" s="14"/>
       <c r="F13" s="7" t="s">
@@ -4890,16 +5457,16 @@
       </c>
       <c r="G13" s="14"/>
       <c r="H13" s="3" t="s">
-        <v>358</v>
+        <v>176</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="7" t="s">
-        <v>359</v>
+        <v>399</v>
       </c>
       <c r="C14" s="14"/>
       <c r="D14" s="7" t="s">
-        <v>204</v>
+        <v>230</v>
       </c>
       <c r="E14" s="14"/>
       <c r="F14" s="7" t="s">
@@ -4907,7 +5474,7 @@
       </c>
       <c r="G14" s="14"/>
       <c r="H14" s="3" t="s">
-        <v>205</v>
+        <v>231</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4917,11 +5484,11 @@
     </row>
     <row r="16" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="7" t="s">
-        <v>360</v>
+        <v>400</v>
       </c>
       <c r="C16" s="14"/>
       <c r="D16" s="7" t="s">
-        <v>361</v>
+        <v>401</v>
       </c>
       <c r="E16" s="14"/>
       <c r="F16" s="7" t="s">
@@ -4938,6 +5505,9 @@
       <c r="G17" s="14"/>
     </row>
     <row r="18" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B18" s="7" t="s">
+        <v>402</v>
+      </c>
       <c r="C18" s="14"/>
       <c r="E18" s="14"/>
       <c r="G18" s="14"/>
@@ -4948,19 +5518,114 @@
       <c r="G19" s="14"/>
     </row>
     <row r="20" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B20" s="7" t="s">
+        <v>403</v>
+      </c>
       <c r="C20" s="14"/>
+      <c r="D20" s="7" t="s">
+        <v>404</v>
+      </c>
       <c r="E20" s="14"/>
+      <c r="F20" s="7" t="s">
+        <v>113</v>
+      </c>
       <c r="G20" s="14"/>
+      <c r="H20" s="3" t="s">
+        <v>405</v>
+      </c>
     </row>
     <row r="21" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B21" s="7" t="s">
+        <v>406</v>
+      </c>
       <c r="C21" s="14"/>
+      <c r="D21" s="7" t="s">
+        <v>407</v>
+      </c>
       <c r="E21" s="14"/>
+      <c r="F21" s="7" t="s">
+        <v>113</v>
+      </c>
       <c r="G21" s="14"/>
+      <c r="H21" s="3" t="s">
+        <v>408</v>
+      </c>
     </row>
     <row r="22" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B22" s="7" t="s">
+        <v>409</v>
+      </c>
       <c r="C22" s="14"/>
+      <c r="D22" s="7" t="s">
+        <v>410</v>
+      </c>
       <c r="E22" s="14"/>
+      <c r="F22" s="7" t="s">
+        <v>113</v>
+      </c>
       <c r="G22" s="14"/>
+      <c r="H22" s="3" t="s">
+        <v>411</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B23" s="7" t="s">
+        <v>412</v>
+      </c>
+      <c r="D23" s="7" t="s">
+        <v>413</v>
+      </c>
+      <c r="F23" s="7" t="s">
+        <v>113</v>
+      </c>
+      <c r="H23" s="3" t="s">
+        <v>414</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B24" s="7" t="s">
+        <v>415</v>
+      </c>
+      <c r="D24" s="7" t="s">
+        <v>416</v>
+      </c>
+      <c r="F24" s="7" t="s">
+        <v>113</v>
+      </c>
+      <c r="H24" s="3" t="s">
+        <v>417</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B25" s="7" t="s">
+        <v>418</v>
+      </c>
+      <c r="C25" s="0"/>
+      <c r="D25" s="7" t="s">
+        <v>419</v>
+      </c>
+      <c r="E25" s="0"/>
+      <c r="F25" s="7" t="s">
+        <v>113</v>
+      </c>
+      <c r="G25" s="0"/>
+      <c r="H25" s="0" t="s">
+        <v>420</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B26" s="7" t="s">
+        <v>421</v>
+      </c>
+      <c r="D26" s="7" t="s">
+        <v>422</v>
+      </c>
+      <c r="F26" s="7" t="s">
+        <v>113</v>
+      </c>
+      <c r="H26" s="3" t="s">
+        <v>423</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -5134,49 +5799,155 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:H18"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="5" min="3" style="7" width="11.53"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="7" min="7" style="7" width="11.53"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="7" width="16.55"/>
+  </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="0" t="s">
-        <v>362</v>
+        <v>424</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="7" t="s">
-        <v>363</v>
+        <v>425</v>
       </c>
       <c r="B3" s="0" t="s">
-        <v>364</v>
+        <v>426</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="7" t="s">
-        <v>365</v>
+        <v>427</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C5" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="D5" s="0" t="s">
-        <v>366</v>
-      </c>
+      <c r="D5" s="7" t="s">
+        <v>428</v>
+      </c>
+      <c r="E5" s="0"/>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C6" s="7" t="n">
+      <c r="E6" s="7" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="F6" s="7" t="s">
+        <v>429</v>
+      </c>
+      <c r="G6" s="7" t="s">
+        <v>430</v>
+      </c>
+      <c r="H6" s="7" t="s">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E7" s="7" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="F7" s="7" t="s">
+        <v>432</v>
+      </c>
+      <c r="G7" s="7" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C8" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="D6" s="0" t="s">
-        <v>367</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C7" s="7" t="n">
+      <c r="D8" s="7" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C9" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="D7" s="0" t="s">
-        <v>368</v>
+      <c r="D9" s="7" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C10" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="D10" s="7" t="s">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C11" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="D11" s="7" t="s">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C12" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="D12" s="7" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C13" s="7" t="n">
+        <v>7</v>
+      </c>
+      <c r="D13" s="7" t="s">
+        <v>439</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C14" s="7" t="n">
+        <v>8</v>
+      </c>
+      <c r="D14" s="7" t="s">
+        <v>440</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C15" s="7" t="n">
+        <v>9</v>
+      </c>
+      <c r="D15" s="7" t="s">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C16" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="D16" s="7" t="s">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C17" s="7" t="n">
+        <v>11</v>
+      </c>
+      <c r="D17" s="7" t="s">
+        <v>443</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C18" s="7" t="n">
+        <v>12</v>
+      </c>
+      <c r="D18" s="7" t="s">
+        <v>444</v>
+      </c>
+      <c r="E18" s="7" t="s">
+        <v>445</v>
       </c>
     </row>
   </sheetData>

</xml_diff>